<commit_message>
chore: fixes, deps, and metadata-template repairs
Repair the metadata-template comment layer + support MSOrganiser v1.x;
guard optional venn/beeswarm plot deps; move ggnewscale to Imports; drop
lifecycle import; strip ANSI in cli colour; roxygen link/Rd sync; stop
tracking generated docs/.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/extdata/metadata_msorganiser_template.xlsx
+++ b/inst/extdata/metadata_msorganiser_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lsibjb/Documents/Code/MRMhub/inst/extdata/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:11_{9D04F58C-11DE-AE4E-AC1D-A526804CC47C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F170AB3-80B9-764C-834C-631FB5D53EEA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="53440" yWindow="20340" windowWidth="67200" windowHeight="21400" tabRatio="624" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="67200" windowHeight="36160" tabRatio="624" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Analyses (Samples)" sheetId="3" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="129">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="130">
   <si>
     <t>ISTD_Conc_[ng/mL]</t>
   </si>
@@ -419,12 +419,6 @@
   </si>
   <si>
     <t>Include_In_Analysis</t>
-  </si>
-  <si>
-    <t>05.06.2026</t>
-  </si>
-  <si>
-    <t>0.2.5</t>
   </si>
   <si>
     <r>
@@ -456,6 +450,15 @@
   </si>
   <si>
     <t>https://github.com/SLINGhub/mrmhub</t>
+  </si>
+  <si>
+    <t>MRM_Pattern</t>
+  </si>
+  <si>
+    <t>1.0.0</t>
+  </si>
+  <si>
+    <t>29.07.2026</t>
   </si>
 </sst>
 </file>
@@ -2253,7 +2256,7 @@
                   <m:sSub>
                     <m:sSubPr>
                       <m:ctrlPr>
-                        <a:rPr lang="en-SG" sz="1600" i="1">
+                        <a:rPr lang="en-US" sz="1600" i="1">
                           <a:effectLst/>
                           <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                           <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
@@ -2302,7 +2305,7 @@
                         <a:rPr lang="en-SG" sz="1600" i="1">
                           <a:effectLst/>
                           <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          <a:ea typeface="DengXian"/>
+                          <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
                           <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
                         </a:rPr>
                       </m:ctrlPr>
@@ -2311,7 +2314,7 @@
                       <m:sSub>
                         <m:sSubPr>
                           <m:ctrlPr>
-                            <a:rPr lang="en-SG" sz="1600" i="1">
+                            <a:rPr lang="en-US" sz="1600" i="1">
                               <a:effectLst/>
                               <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                               <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
@@ -2350,7 +2353,7 @@
                       <m:sSub>
                         <m:sSubPr>
                           <m:ctrlPr>
-                            <a:rPr lang="en-SG" sz="1600" i="1">
+                            <a:rPr lang="en-US" sz="1600" i="1">
                               <a:effectLst/>
                               <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
                               <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
@@ -2399,10 +2402,13 @@
                     <m:fPr>
                       <m:ctrlPr>
                         <a:rPr lang="en-SG" sz="1600" i="1">
+                          <a:solidFill>
+                            <a:schemeClr val="dk1"/>
+                          </a:solidFill>
                           <a:effectLst/>
                           <a:latin typeface="Cambria Math" panose="02040503050406030204" pitchFamily="18" charset="0"/>
-                          <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-                          <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
+                          <a:ea typeface="+mn-ea"/>
+                          <a:cs typeface="+mn-cs"/>
                         </a:rPr>
                       </m:ctrlPr>
                     </m:fPr>
@@ -2410,7 +2416,7 @@
                       <m:sSub>
                         <m:sSubPr>
                           <m:ctrlPr>
-                            <a:rPr lang="en-SG" sz="1600" i="1">
+                            <a:rPr lang="en-US" sz="1600" b="0" i="1">
                               <a:solidFill>
                                 <a:schemeClr val="dk1"/>
                               </a:solidFill>
@@ -7104,7 +7110,7 @@
   <sheetPr codeName="TransitionNameAnnotSheet">
     <tabColor theme="4" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:O10"/>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.1640625" defaultRowHeight="19" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="31.33203125" style="20" customWidth="1"/>
@@ -7116,14 +7122,15 @@
     <col min="8" max="8" width="21.5" style="20" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="14.5" style="20" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="24.1640625" style="20" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="35.1640625" style="20" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="32.5" style="20" bestFit="1" customWidth="1"/>
-    <col min="13" max="14" width="32.5" style="20" customWidth="1"/>
-    <col min="15" max="15" width="10.5" style="20" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="9.1640625" style="13"/>
+    <col min="11" max="11" width="24.1640625" style="20" customWidth="1"/>
+    <col min="12" max="12" width="35.1640625" style="20" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="32.5" style="20" bestFit="1" customWidth="1"/>
+    <col min="14" max="15" width="32.5" style="20" customWidth="1"/>
+    <col min="16" max="16" width="10.5" style="20" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="9.1640625" style="13"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" s="32" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:16" s="32" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="37" t="s">
         <v>79</v>
       </c>
@@ -7155,43 +7162,46 @@
         <v>81</v>
       </c>
       <c r="K1" s="31" t="s">
+        <v>127</v>
+      </c>
+      <c r="L1" s="31" t="s">
         <v>94</v>
       </c>
-      <c r="L1" s="31" t="s">
+      <c r="M1" s="31" t="s">
         <v>95</v>
       </c>
-      <c r="M1" s="60" t="s">
+      <c r="N1" s="60" t="s">
         <v>120</v>
       </c>
-      <c r="N1" s="60" t="s">
+      <c r="O1" s="60" t="s">
         <v>121</v>
       </c>
-      <c r="O1" s="31" t="s">
+      <c r="P1" s="31" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3" s="13"/>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4" s="13"/>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5" s="13"/>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6" s="13"/>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7" s="13"/>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8" s="13"/>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9" s="13"/>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10" s="13"/>
     </row>
   </sheetData>
@@ -8724,7 +8734,7 @@
         <v>92</v>
       </c>
       <c r="C3" s="56" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="D3" s="43"/>
     </row>
@@ -8734,7 +8744,7 @@
         <v>91</v>
       </c>
       <c r="C4" s="52" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="D4" s="28"/>
     </row>
@@ -8747,7 +8757,7 @@
     <row r="6" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="29"/>
       <c r="B6" s="52" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C6" s="52"/>
       <c r="D6" s="29"/>
@@ -8769,7 +8779,7 @@
     <row r="9" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A9" s="38"/>
       <c r="B9" s="38" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C9" s="52"/>
       <c r="D9" s="29"/>
@@ -8780,7 +8790,7 @@
         <v>115</v>
       </c>
       <c r="C10" s="59" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="D10" s="29"/>
     </row>
@@ -8833,7 +8843,7 @@
     <row r="17" spans="1:4" ht="16" x14ac:dyDescent="0.2">
       <c r="A17" s="29"/>
       <c r="B17" s="38" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C17" s="52"/>
       <c r="D17" s="29"/>
@@ -8857,6 +8867,7 @@
       <c r="D20" s="29"/>
     </row>
   </sheetData>
+  <sheetProtection sheet="1" objects="1" scenarios="1"/>
   <phoneticPr fontId="32" type="noConversion"/>
   <hyperlinks>
     <hyperlink ref="B13" r:id="rId1" xr:uid="{B5F9473A-8279-DA49-9BBC-7EE864686E47}"/>
@@ -8869,9 +8880,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -9013,26 +9027,15 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F7782B24-6BC4-4055-A0EF-8E7D4305C5AF}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AD972C8C-3C83-494C-96B6-0C830C869D3F}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="e63a464c-78f9-4e2d-a62f-b57ec6de9f3d"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -9056,9 +9059,17 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AD972C8C-3C83-494C-96B6-0C830C869D3F}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F7782B24-6BC4-4055-A0EF-8E7D4305C5AF}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="e63a464c-78f9-4e2d-a62f-b57ec6de9f3d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>